<commit_message>
Structured group and second peer review, clarified day 2 of week 3.
</commit_message>
<xml_diff>
--- a/peer_review/20260522_du_jufe_dm_peer_review_02_vector_student.xlsx
+++ b/peer_review/20260522_du_jufe_dm_peer_review_02_vector_student.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rpi\source\20260512_du_jufe_dm\20260512_du_jufe_dm_rpi\peer_review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{4822FBA1-48A0-4431-AE42-58DACCD1C84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4D4435-CA66-4FD7-A7A1-4215333E3B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{71A9985A-D91F-47EE-BF6E-5C7AC9C1D4EE}"/>
   </bookViews>
@@ -683,14 +683,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % - Dekorfärg1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1085,7 +1083,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1101,24 +1099,24 @@
       <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="5">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="C3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F3">
@@ -1126,19 +1124,19 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="C4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F4">
@@ -1146,19 +1144,19 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="5">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="C5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>12</v>
       </c>
       <c r="F5">
@@ -1166,19 +1164,19 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="5">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="C6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F6">
@@ -1186,19 +1184,19 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="5">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="C7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="4" t="s">
         <v>16</v>
       </c>
       <c r="F7">
@@ -1206,19 +1204,19 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="5">
-        <v>6</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="5" t="s">
+      <c r="C8" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="4" t="s">
         <v>18</v>
       </c>
       <c r="F8">
@@ -1226,19 +1224,19 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
+      <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="C9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F9">

</xml_diff>